<commit_message>
Day 5 - Scenario 4
</commit_message>
<xml_diff>
--- a/Sprint/PractoTesting/src/test/resource/Exceldata/LabTestData.xlsx
+++ b/Sprint/PractoTesting/src/test/resource/Exceldata/LabTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SDHINDLE\Desktop\PRACTO\Sprint\PractoTesting\src\test\resource\Exceldata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E100129E-AE24-47A5-9BF1-7F9BE49EDB0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{104DD8F8-4C65-4399-B2F3-2FF41BBEE3FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>username</t>
   </si>
@@ -43,6 +43,24 @@
   </si>
   <si>
     <t>+917066798939</t>
+  </si>
+  <si>
+    <t>patientName</t>
+  </si>
+  <si>
+    <t>patientAge</t>
+  </si>
+  <si>
+    <t>patientEmail</t>
+  </si>
+  <si>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>alice@gmail.com</t>
+  </si>
+  <si>
+    <t>21</t>
   </si>
 </sst>
 </file>
@@ -372,13 +390,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.26953125" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="11.453125" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -388,8 +409,17 @@
       <c r="C1" t="s">
         <v>3</v>
       </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -398,11 +428,21 @@
       </c>
       <c r="C2" t="s">
         <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{C9E9898C-9814-475E-9324-A713D6D7EAE8}"/>
+    <hyperlink ref="F2" r:id="rId2" xr:uid="{57CD8176-3774-4878-9CE3-1B2095059A15}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>